<commit_message>
added scripts folder, updated logs
</commit_message>
<xml_diff>
--- a/Research Logs/Matt/Matt Baker - Week 10 Research Log.xlsx
+++ b/Research Logs/Matt/Matt Baker - Week 10 Research Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Research Logs\Matt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF0C2AE-F97B-4C1E-BFF4-6DCAFAB96B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4130E1-959E-44E7-AAA0-9BF2070EECFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="142">
   <si>
     <t>Date</t>
   </si>
@@ -495,6 +495,50 @@
   </si>
   <si>
     <t>The guy demonstrates that you can convert pcaps to JSON to make them ingestible to chatgpt, so this gives me something to test with ollama integration. His resulkts show chatgpt was unable to idscover the source of slow network traffic in the pcap, but gemini was able to give an undistracted analysis. It was interesting to see his perspective as a professional wireshark analyst on the outcome.</t>
+  </si>
+  <si>
+    <t>Why does AI prefer JSON format to determine if that if an input format I should work with</t>
+  </si>
+  <si>
+    <t>I found out that JSON is used because of it's strict structure, it makes it easier for AI to digest for prompts, for me, my prompts arent advanced enough and my data cant be converted realistically into json format, although existing tools for converting pcaps to JSON will be looked into later</t>
+  </si>
+  <si>
+    <t>Google
+https://www.w3schools.com/JS/js_json.asp
+https://demiliani.com/2025/08/07/json-prompting-in-ai-why/</t>
+  </si>
+  <si>
+    <t>What Ollama statistics mean (prompt_eval/eval count, duration, and rate), this requires learning
+a bit more about tokens themselves</t>
+  </si>
+  <si>
+    <t>Ollama documentation was useful, prompt_eval_count seems to be the token size of the prompt in tokens, and eval_count is the size of the output in tokens. Both input and output tokens add up to the total context window.</t>
+  </si>
+  <si>
+    <t>Google
+https://docs.ollama.com/api/usage
+https://learn.microsoft.com/en-us/dotnet/ai/conceptual/understanding-tokens</t>
+  </si>
+  <si>
+    <t>How to convert nmap Pcap files to JSON, find existing solutions</t>
+  </si>
+  <si>
+    <t>https://github.com/D4-project/nmap2json
+https://gist.github.com/PSJoshi/c2f1bacfff3d18f39203920335a66828</t>
+  </si>
+  <si>
+    <t>NmaptoJSON is the better solution for our purpose as it can just be called from command line, although it requires a virtual environment. I had to read the documentation to figure out how to get it to work.</t>
+  </si>
+  <si>
+    <t>How to convert string to float to save metrics from ollama verbose output and add them</t>
+  </si>
+  <si>
+    <t>https://stackoverflow.com/questions/4703390/how-to-extract-a-floating-number-from-a-string
+https://stackoverflow.com/questions/4289331/how-to-extract-numbers-from-a-string-in-python
+https://www.w3schools.com/python/ref_module_re.asp</t>
+  </si>
+  <si>
+    <t>Some tinkering of these script examples and understanding of the re.findall syntax used to identify specific data following strings helped me eventually extract integers (token counts) from the --verbose output</t>
   </si>
 </sst>
 </file>
@@ -863,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G55"/>
+  <dimension ref="B2:G59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" style="3" customWidth="1"/>
@@ -880,7 +924,7 @@
       </c>
       <c r="D2" s="5">
         <f>ROUNDDOWN(SUM(C6:C499)/60,0)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -892,7 +936,7 @@
       </c>
       <c r="D3" s="5">
         <f>ROUND(MOD(SUM(C6:C499),60),0)</f>
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -1671,6 +1715,86 @@
       </c>
       <c r="G55" s="1" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="B56" s="3">
+        <v>46281</v>
+      </c>
+      <c r="C56">
+        <v>45</v>
+      </c>
+      <c r="D56" t="s">
+        <v>43</v>
+      </c>
+      <c r="E56" t="s">
+        <v>130</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B57" s="3">
+        <v>46281</v>
+      </c>
+      <c r="C57">
+        <v>30</v>
+      </c>
+      <c r="D57" t="s">
+        <v>43</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B58" s="3">
+        <v>46284</v>
+      </c>
+      <c r="C58">
+        <v>30</v>
+      </c>
+      <c r="D58" t="s">
+        <v>57</v>
+      </c>
+      <c r="E58" t="s">
+        <v>136</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B59" s="3">
+        <v>46284</v>
+      </c>
+      <c r="C59">
+        <v>30</v>
+      </c>
+      <c r="D59" t="s">
+        <v>14</v>
+      </c>
+      <c r="E59" t="s">
+        <v>139</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1692,6 +1816,8 @@
     <hyperlink ref="G45" r:id="rId15" xr:uid="{D120BCEA-4978-4ECC-9CD1-F5B933D36DD0}"/>
     <hyperlink ref="G46" r:id="rId16" display="https://deepseek-harness.github.io/deepseek-harness/en/guide/quickstart" xr:uid="{139F3B52-FE4E-48B5-818F-8B1AC93CD598}"/>
     <hyperlink ref="G51" r:id="rId17" display="https://www.youtube.com/watch?v=2Fp1N6dof0Y" xr:uid="{8B5A1D2F-2AA3-4DEF-8372-4C8C97A9C922}"/>
+    <hyperlink ref="G58" r:id="rId18" display="https://github.com/D4-project/nmap2json" xr:uid="{C857808A-F7DD-4DA4-B603-3F21024AF8C8}"/>
+    <hyperlink ref="G59" r:id="rId19" display="https://stackoverflow.com/questions/4703390/how-to-extract-a-floating-number-from-a-string" xr:uid="{42FBAB5B-B3FE-4D89-B36B-858373BD4E7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>